<commit_message>
Docs: update BOM and fix Pin Map
</commit_message>
<xml_diff>
--- a/hardware/bom/BOM_V0.1_with_PinMap.xlsx
+++ b/hardware/bom/BOM_V0.1_with_PinMap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DOWNLOAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E09FAD21-6CFF-43AF-B720-86E8CF421BA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7742C55-B76D-4F42-8168-2BD2BEEA1D48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,14 +17,14 @@
     <sheet name="Quy hoach chan ESP32-S3" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Quy hoach chan ESP32-S3'!$A$3:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Quy hoach chan ESP32-S3'!$A$3:$G$15</definedName>
   </definedNames>
   <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="83">
   <si>
     <t>BOM v0.1 (Thiết bị đo huyết áp không vòng bít PPG/ECG (Bản v0 – bản thí nghiệm)</t>
   </si>
@@ -62,15 +62,6 @@
     <t>ECG AFE</t>
   </si>
   <si>
-    <t>ProtoCentral MAX30001 breakout (SPI, ECG + BioZ)</t>
-  </si>
-  <si>
-    <t>ProtoCentral ADS1292R breakout (có RLD, 500 SPS, kèm điện cực/cáp); MAX30003</t>
-  </si>
-  <si>
-    <t>MAX30001 là ECG AFE chuyên dụng, phù hợp mục tiêu thu ECG chất lượng và kiểm chứng AFE trước khi thiết kế phần cứng riêng</t>
-  </si>
-  <si>
     <t>MCU</t>
   </si>
   <si>
@@ -89,9 +80,6 @@
     <t>Điện cực dán Ag/AgCl 3M Red Dot 2228</t>
   </si>
   <si>
-    <t>Điện cực đi kèm với max30001</t>
-  </si>
-  <si>
     <t>Dễ mua, phù hợp với dự án ở tiến độ hiện tại</t>
   </si>
   <si>
@@ -152,93 +140,18 @@
     <t>Trạng thái</t>
   </si>
   <si>
-    <t>Ghi chú</t>
-  </si>
-  <si>
-    <t>MAX30001</t>
-  </si>
-  <si>
-    <t>GPIO13 (FSPIQ)</t>
-  </si>
-  <si>
-    <t>SPI</t>
-  </si>
-  <si>
-    <t>MAX30001 → ESP32-S3</t>
-  </si>
-  <si>
     <t>Đề xuất</t>
   </si>
   <si>
-    <t>FSPIQ là đường dữ liệu vào của SPI Master; nhận dữ liệu từ SDO.</t>
-  </si>
-  <si>
-    <t>GPIO11 (FSPID)</t>
-  </si>
-  <si>
-    <t>ESP32-S3 → MAX30001</t>
-  </si>
-  <si>
-    <t>FSPID là đường dữ liệu ra của SPI Master; gửi dữ liệu tới SDI.</t>
-  </si>
-  <si>
-    <t>SCK</t>
-  </si>
-  <si>
-    <t>GPIO12 (FSPICLK)</t>
-  </si>
-  <si>
-    <t>Clock SPI do ESP32-S3 tạo.</t>
-  </si>
-  <si>
-    <t>GPIO10 (FSPICS0)</t>
-  </si>
-  <si>
-    <t>CS active-low: kéo LOW để chọn MAX30001.</t>
-  </si>
-  <si>
-    <t>INT1</t>
-  </si>
-  <si>
     <t>GPIO5</t>
   </si>
   <si>
-    <t>GPIO/INT</t>
-  </si>
-  <si>
-    <t>Ngắt báo sự kiện/dữ liệu; cần kiểm tra cấu hình INT trong firmware.</t>
-  </si>
-  <si>
-    <t>INT2</t>
-  </si>
-  <si>
     <t>Chưa dùng</t>
   </si>
   <si>
-    <t>Không nối trong cấu hình V0 cơ bản.</t>
-  </si>
-  <si>
-    <t>FCLK</t>
-  </si>
-  <si>
-    <t>Clock</t>
-  </si>
-  <si>
-    <t>Không nối trong cấu hình V0 cơ bản; dùng clock nội bộ theo cấu hình breakout.</t>
-  </si>
-  <si>
-    <t>VCC</t>
-  </si>
-  <si>
-    <t>Power</t>
-  </si>
-  <si>
     <t>GND</t>
   </si>
   <si>
-    <t>Mass chung giữa ESP32-S3 và breakout.</t>
-  </si>
-  <si>
     <t>ECGP / ECGN / RL</t>
   </si>
   <si>
@@ -248,88 +161,118 @@
     <t>ECG</t>
   </si>
   <si>
-    <t>Điện cực → MAX30001</t>
-  </si>
-  <si>
-    <t>Điện cực không nối trực tiếp vào GPIO ESP32-S3.</t>
-  </si>
-  <si>
-    <t>PPG AFE (chưa chốt)</t>
-  </si>
-  <si>
     <t>SDA</t>
   </si>
   <si>
-    <t>GPIO1</t>
-  </si>
-  <si>
     <t>I2C</t>
   </si>
   <si>
-    <t>Hai chiều</t>
-  </si>
-  <si>
-    <t>Pin dự kiến theo quy hoạch hiện tại; PPG AFE chưa được chốt trong BOM.</t>
-  </si>
-  <si>
     <t>SCL</t>
   </si>
   <si>
-    <t>GPIO2</t>
-  </si>
-  <si>
-    <t>ESP32-S3 → PPG AFE</t>
-  </si>
-  <si>
-    <t>Pin dự kiến theo quy hoạch hiện tại; kiểm tra pull-up 3.3 V.</t>
-  </si>
-  <si>
     <t>INT</t>
   </si>
   <si>
     <t>GPIO4</t>
   </si>
   <si>
-    <t>PPG AFE → ESP32-S3</t>
-  </si>
-  <si>
-    <t>Chỉ dùng nếu breakout/AFE có chân INT và firmware cần.</t>
-  </si>
-  <si>
     <t>Ghi chú quan trọng</t>
   </si>
   <si>
-    <t>• ESP32-S3 là SPI Master; MAX30001 là SPI Slave.</t>
-  </si>
-  <si>
-    <t>• Mapping SPI hiện tại: GPIO11 = FSPID/MOSI, GPIO12 = FSPICLK/SCK, GPIO13 = FSPIQ/MISO, GPIO10 = FSPICS0/CS.</t>
-  </si>
-  <si>
-    <t>• Không nối nhầm MOSI/MISO: Master MOSI → Slave SDI; Master MISO ← Slave SDO.</t>
-  </si>
-  <si>
-    <t>• PPG AFE chưa được chốt trong BOM, vì vậy các chân GPIO1/GPIO2/GPIO4 chỉ là quy hoạch dự kiến.</t>
-  </si>
-  <si>
     <t>• Pin map cần kiểm tra lại khi đi dây thực tế và sau khi đọc datasheet/breakout pinout của linh kiện được duyệt.</t>
   </si>
   <si>
-    <t xml:space="preserve">MISO </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MOSI </t>
-  </si>
-  <si>
-    <t>CS0</t>
-  </si>
-  <si>
     <t>ESP32_S3 → MAX30001</t>
   </si>
   <si>
-    <t>Breakout ProtoCentral hỗ trợ VCC 3.3 V hoặc 5 V</t>
-  </si>
-  <si>
-    <t>3V3 hoặc 5V0</t>
+    <t>Module MAX30102</t>
+  </si>
+  <si>
+    <t>Module Max30100</t>
+  </si>
+  <si>
+    <t>ProtoCentral Max30001 breakout</t>
+  </si>
+  <si>
+    <t>Module ECG AD8232</t>
+  </si>
+  <si>
+    <t>Điện cực đi kèm với set của AD8232</t>
+  </si>
+  <si>
+    <t>Dễ mua, phù hợp với bản V0</t>
+  </si>
+  <si>
+    <t>Lí do lựa chọn</t>
+  </si>
+  <si>
+    <t>Dễ mua, phù hợp với bản V0, đáp ứng đủ yêu cầu ở phiên bản hiện tại</t>
+  </si>
+  <si>
+    <t>AD8232</t>
+  </si>
+  <si>
+    <t>OUTPUT</t>
+  </si>
+  <si>
+    <t>Analog -&gt; ADC</t>
+  </si>
+  <si>
+    <t>AD8232 → ESP32-S3</t>
+  </si>
+  <si>
+    <t>3.3V</t>
+  </si>
+  <si>
+    <t>3V3</t>
+  </si>
+  <si>
+    <t>POWER</t>
+  </si>
+  <si>
+    <t>ESP32-S3 → AD8232</t>
+  </si>
+  <si>
+    <t>LO+</t>
+  </si>
+  <si>
+    <t>Digital GPIO</t>
+  </si>
+  <si>
+    <t>LO-</t>
+  </si>
+  <si>
+    <t>GPIO6</t>
+  </si>
+  <si>
+    <t>SDN</t>
+  </si>
+  <si>
+    <t>MAX30102</t>
+  </si>
+  <si>
+    <t>VIN</t>
+  </si>
+  <si>
+    <t>ESP32-S3 -&gt; MAX30102</t>
+  </si>
+  <si>
+    <t>GPIO8</t>
+  </si>
+  <si>
+    <t>MAX30102 -&gt; ESP32-S3</t>
+  </si>
+  <si>
+    <t>Điện cực → MAX30102</t>
+  </si>
+  <si>
+    <t>GPIO9</t>
+  </si>
+  <si>
+    <t>GPIO10</t>
+  </si>
+  <si>
+    <t>MAX30102 → ESP32-S3</t>
   </si>
 </sst>
 </file>
@@ -758,7 +701,9 @@
       <c r="D3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>59</v>
+      </c>
       <c r="F3" s="2" t="s">
         <v>5</v>
       </c>
@@ -776,9 +721,15 @@
       <c r="B4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
+      <c r="C4" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>58</v>
+      </c>
       <c r="F4" s="3" t="s">
         <v>9</v>
       </c>
@@ -797,13 +748,13 @@
         <v>11</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>12</v>
+        <v>56</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>13</v>
+        <v>55</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>9</v>
@@ -820,16 +771,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>9</v>
@@ -846,22 +797,22 @@
         <v>4</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>20</v>
+        <v>57</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>9</v>
       </c>
       <c r="G7" s="4">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>10</v>
@@ -872,19 +823,19 @@
         <v>5</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>27</v>
       </c>
       <c r="G8" s="4">
         <v>2</v>
@@ -898,20 +849,20 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3" t="s">
         <v>9</v>
       </c>
       <c r="G9" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>10</v>
@@ -922,13 +873,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3" t="s">
@@ -946,20 +897,20 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>32</v>
-      </c>
       <c r="D11" s="3" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3" t="s">
         <v>9</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>10</v>
@@ -979,7 +930,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -988,12 +939,11 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="25" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="65" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -1001,446 +951,305 @@
       <c r="E1" s="9"/>
       <c r="F1" s="9"/>
       <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-    </row>
-    <row r="3" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="6">
         <v>1</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>96</v>
+        <v>62</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="6">
         <v>2</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>43</v>
-      </c>
+      <c r="B5" s="6"/>
       <c r="C5" s="6" t="s">
-        <v>97</v>
+        <v>65</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="6">
         <v>3</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>43</v>
-      </c>
+      <c r="B6" s="6"/>
       <c r="C6" s="6" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="6">
         <v>4</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>43</v>
-      </c>
+      <c r="B7" s="6"/>
       <c r="C7" s="6" t="s">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="6">
         <v>5</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>43</v>
-      </c>
+      <c r="B8" s="6"/>
       <c r="C8" s="6" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="6">
         <v>6</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>43</v>
-      </c>
+      <c r="B9" s="6"/>
       <c r="C9" s="6" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>59</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="E9" s="6"/>
       <c r="F9" s="6" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="6">
         <v>7</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>43</v>
+        <v>74</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>30</v>
+        <v>66</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>30</v>
+        <v>76</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="6">
         <v>8</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>43</v>
-      </c>
+      <c r="B11" s="6"/>
       <c r="C11" s="6" t="s">
-        <v>67</v>
+        <v>41</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>101</v>
+        <v>41</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>68</v>
+        <v>41</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>99</v>
+        <v>52</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="6">
         <v>9</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>43</v>
-      </c>
+      <c r="B12" s="6"/>
       <c r="C12" s="6" t="s">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>68</v>
+        <v>46</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="6">
         <v>10</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="6"/>
+      <c r="C13" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>72</v>
-      </c>
       <c r="E13" s="6" t="s">
-        <v>73</v>
+        <v>44</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G13" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H13" s="6" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="6">
         <v>11</v>
       </c>
-      <c r="B14" s="6" t="s">
-        <v>76</v>
-      </c>
+      <c r="B14" s="6"/>
       <c r="C14" s="6" t="s">
-        <v>77</v>
+        <v>47</v>
       </c>
       <c r="D14" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="F14" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="E14" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>80</v>
-      </c>
       <c r="G14" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="6">
         <v>12</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>76</v>
-      </c>
+      <c r="B15" s="6"/>
       <c r="C15" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D15" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>84</v>
-      </c>
       <c r="G15" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="6">
-        <v>13</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="7" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A21" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="B21" s="9"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="B22" s="9"/>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A23" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="B23" s="9"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A24" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H16" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
-  <mergeCells count="6">
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A24:H24"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="A22:H22"/>
+  <autoFilter ref="A3:G15" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <mergeCells count="2">
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>